<commit_message>
fix(config): 直充钻石改整十（1130/2380/8420）+ CRC 同步 + retune 常量对齐
</commit_message>
<xml_diff>
--- a/data_execl/base_data/RechargeCommodityConfig.xlsx
+++ b/data_execl/base_data/RechargeCommodityConfig.xlsx
@@ -21494,17 +21494,17 @@
       </c>
       <c r="K259" s="0" t="inlineStr">
         <is>
-          <t>16#1127</t>
+          <t>16#1130</t>
         </is>
       </c>
       <c r="L259" s="0" t="inlineStr">
         <is>
-          <t>16#1127|6000124#980</t>
+          <t>16#1130|6000124#980</t>
         </is>
       </c>
       <c r="M259" s="0" t="inlineStr">
         <is>
-          <t>16#1127</t>
+          <t>16#1130</t>
         </is>
       </c>
       <c r="Q259" s="0" t="n">
@@ -21577,17 +21577,17 @@
       </c>
       <c r="K260" s="0" t="inlineStr">
         <is>
-          <t>16#2376</t>
+          <t>16#2380</t>
         </is>
       </c>
       <c r="L260" s="0" t="inlineStr">
         <is>
-          <t>16#2376|6000124#1980</t>
+          <t>16#2380|6000124#1980</t>
         </is>
       </c>
       <c r="M260" s="0" t="inlineStr">
         <is>
-          <t>16#2376</t>
+          <t>16#2380</t>
         </is>
       </c>
       <c r="Q260" s="0" t="n">
@@ -21743,17 +21743,17 @@
       </c>
       <c r="K262" s="0" t="inlineStr">
         <is>
-          <t>16#8424</t>
+          <t>16#8420</t>
         </is>
       </c>
       <c r="L262" s="0" t="inlineStr">
         <is>
-          <t>16#8424|6000124#6480</t>
+          <t>16#8420|6000124#6480</t>
         </is>
       </c>
       <c r="M262" s="0" t="inlineStr">
         <is>
-          <t>16#8424</t>
+          <t>16#8420</t>
         </is>
       </c>
       <c r="Q262" s="0" t="n">

</xml_diff>